<commit_message>
Tidy sheet names in NBRK monthly workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017voBJECUQYsPVYf3NcKDQ7
</commit_message>
<xml_diff>
--- a/bank_analysis/out/NBRK_banki_2026_po_mesyacam.xlsx
+++ b/bank_analysis/out/NBRK_banki_2026_po_mesyacam.xlsx
@@ -8,18 +8,18 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прибыль по месяцам" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Активы млрд тг" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ссудный портфель млрд тг" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Собственный капитал по балансу" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Чистая прибыль с начала года м" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Просрочка &gt;90 дней pct портфеля" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Кредиты 3 стадии и ПСКО % порт" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Провизии по ссудному портфелю " sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="k1 pct" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="k1-2 pct" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="k2 pct" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процентная маржа (НБРК) pct" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процентный спред pct" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Активы (млрд тг)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Кредиты (млрд тг)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Капитал (млрд тг)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ЧП с начала года (млрд тг)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Просрочка 90+ (%)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stage 3 и ПСКО (%)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Провизии (млрд тг)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="k1 (%)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="k1-2 (%)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="k2 (%)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процентная маржа (%)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процентный спред (%)" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>